<commit_message>
script_migration_stock_config: [UPG] Migration Script 2
</commit_message>
<xml_diff>
--- a/script_migration_stock_config/static/data/Inventory Adj (stock.location).xlsx
+++ b/script_migration_stock_config/static/data/Inventory Adj (stock.location).xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/waiyan/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/waiyan/Project/Odoo/ppg/ppg/ppg/ppg/script_migration_stock_config/static/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BE7E429-FF4D-9D4D-B620-2BDB7BBF1B2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85FE6C7B-2541-6D44-917A-FEF50D268AAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="80" yWindow="660" windowWidth="30160" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2623,17 +2623,17 @@
       <c r="C193" s="2"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A1:A113 A115:A1048576">
+    <cfRule type="duplicateValues" dxfId="3" priority="10"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A114">
-    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B1:B113 B115:B1048576">
+    <cfRule type="duplicateValues" dxfId="1" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B114">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A1:A113 A115:A1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="10"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B1:B113 B115:B1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>